<commit_message>
Add Bangkok attraction fees to v0.9 interim workbook
</commit_message>
<xml_diff>
--- a/GPT전달내용/travel_cost_research_pilot_v0.9_2026-10-03.xlsx
+++ b/GPT전달내용/travel_cost_research_pilot_v0.9_2026-10-03.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조사 기준" sheetId="1" r:id="Rb6f9cdde0bc44b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 우선순위" sheetId="2" r:id="R2114cbcbfe8440ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가격 표본" sheetId="3" r:id="Rb3f1b7b6cd6d48ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="음식 추천" sheetId="4" r:id="R07dafe6b4a5048d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 초안" sheetId="5" r:id="R03c8853319054687"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다음 조사 큐" sheetId="6" r:id="R0bf91b811e1e4674"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조사 기준" sheetId="1" r:id="R84a71f58c7164a18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 우선순위" sheetId="2" r:id="Rd0d7e45a14b3486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가격 표본" sheetId="3" r:id="Re1f3a245c39544bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="음식 추천" sheetId="4" r:id="R06141027e1f34b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도시 초안" sheetId="5" r:id="Ra4666ae008ce4979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다음 조사 큐" sheetId="6" r:id="R56e12de9f2ab4999"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -334,8 +334,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriceObservationTable" displayName="PriceObservationTable" ref="A4:U293" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:U293"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriceObservationTable" displayName="PriceObservationTable" ref="A4:U308" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:U308"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="국가"/>
@@ -1796,7 +1796,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref0fb08204164e58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8db1de4475411f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20691,6 +20691,981 @@
         <x:v>공원 공식 안내의 중학생 이하 무료 입장.</x:v>
       </x:c>
     </x:row>
+    <x:row r="294" ht="36" customHeight="1">
+      <x:c r="A294" t="str">
+        <x:v>BKK-AT-004</x:v>
+      </x:c>
+      <x:c r="B294" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C294" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D294" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E294" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F294" t="str">
+        <x:v>짐 톰슨 하우스 박물관 성인 입장권</x:v>
+      </x:c>
+      <x:c r="G294" t="str">
+        <x:v>Jim Thompson House Museum Adult Admission</x:v>
+      </x:c>
+      <x:c r="H294" s="55" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="I294" s="55" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="J294" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K294" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L294" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M294" t="str">
+        <x:v>성인 22세 이상</x:v>
+      </x:c>
+      <x:c r="N294" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O294" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P294" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q294" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R294" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S294" t="str">
+        <x:v>The Jim Thompson House Museum</x:v>
+      </x:c>
+      <x:c r="T294" t="str">
+        <x:v>https://jimthompsonhouse.org/</x:v>
+      </x:c>
+      <x:c r="U294" s="23" t="str">
+        <x:v>박물관 공식 안내의 성인 입장료 250바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="295" ht="36" customHeight="1">
+      <x:c r="A295" t="str">
+        <x:v>BKK-AT-005</x:v>
+      </x:c>
+      <x:c r="B295" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C295" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D295" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E295" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F295" t="str">
+        <x:v>짐 톰슨 하우스 박물관 10~21세 입장권</x:v>
+      </x:c>
+      <x:c r="G295" t="str">
+        <x:v>Jim Thompson House Museum Admission (Age 10-21)</x:v>
+      </x:c>
+      <x:c r="H295" s="55" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="I295" s="55" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="J295" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K295" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L295" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M295" t="str">
+        <x:v>10~21세 (신분증 제시)</x:v>
+      </x:c>
+      <x:c r="N295" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O295" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P295" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q295" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R295" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S295" t="str">
+        <x:v>The Jim Thompson House Museum</x:v>
+      </x:c>
+      <x:c r="T295" t="str">
+        <x:v>https://jimthompsonhouse.org/</x:v>
+      </x:c>
+      <x:c r="U295" s="23" t="str">
+        <x:v>박물관 공식 안내의 10~21세 요금 150바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="36" customHeight="1">
+      <x:c r="A296" t="str">
+        <x:v>BKK-AT-006</x:v>
+      </x:c>
+      <x:c r="B296" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C296" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D296" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E296" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F296" t="str">
+        <x:v>짐 톰슨 하우스 박물관 10세 미만 무료 입장</x:v>
+      </x:c>
+      <x:c r="G296" t="str">
+        <x:v>Jim Thompson House Museum Free Admission (Under 10)</x:v>
+      </x:c>
+      <x:c r="H296" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I296" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J296" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K296" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L296" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M296" t="str">
+        <x:v>10세 미만 (성인 동반)</x:v>
+      </x:c>
+      <x:c r="N296" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O296" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P296" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q296" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R296" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S296" t="str">
+        <x:v>The Jim Thompson House Museum</x:v>
+      </x:c>
+      <x:c r="T296" t="str">
+        <x:v>https://jimthompsonhouse.org/</x:v>
+      </x:c>
+      <x:c r="U296" s="23" t="str">
+        <x:v>박물관 공식 안내의 성인 동반 10세 미만 무료 입장.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="36" customHeight="1">
+      <x:c r="A297" t="str">
+        <x:v>BKK-AT-007</x:v>
+      </x:c>
+      <x:c r="B297" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C297" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D297" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E297" t="str">
+        <x:v>전망대</x:v>
+      </x:c>
+      <x:c r="F297" t="str">
+        <x:v>마하나콘 스카이워크 성인 입장권</x:v>
+      </x:c>
+      <x:c r="G297" t="str">
+        <x:v>Mahanakhon SkyWalk Adult Admission</x:v>
+      </x:c>
+      <x:c r="H297" s="55" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I297" s="55" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J297" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K297" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L297" t="str">
+        <x:v>수요형</x:v>
+      </x:c>
+      <x:c r="M297" t="str">
+        <x:v>성인 13세 이상</x:v>
+      </x:c>
+      <x:c r="N297" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O297" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P297" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q297" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R297" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S297" t="str">
+        <x:v>King Power Mahanakhon</x:v>
+      </x:c>
+      <x:c r="T297" t="str">
+        <x:v>https://kingpowermahanakhon.co.th/th/experience/mahanakhon-skywalk</x:v>
+      </x:c>
+      <x:c r="U297" s="23" t="str">
+        <x:v>운영사 공식 안내의 성인권은 10:00~15:30 1,000바트, 15:30~19:00 1,200바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="36" customHeight="1">
+      <x:c r="A298" t="str">
+        <x:v>BKK-AT-008</x:v>
+      </x:c>
+      <x:c r="B298" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C298" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D298" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E298" t="str">
+        <x:v>전망대</x:v>
+      </x:c>
+      <x:c r="F298" t="str">
+        <x:v>마하나콘 스카이워크 어린이 입장권</x:v>
+      </x:c>
+      <x:c r="G298" t="str">
+        <x:v>Mahanakhon SkyWalk Child Admission</x:v>
+      </x:c>
+      <x:c r="H298" s="55" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I298" s="55" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="J298" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K298" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L298" t="str">
+        <x:v>수요형</x:v>
+      </x:c>
+      <x:c r="M298" t="str">
+        <x:v>3~12세</x:v>
+      </x:c>
+      <x:c r="N298" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O298" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P298" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q298" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R298" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S298" t="str">
+        <x:v>King Power Mahanakhon</x:v>
+      </x:c>
+      <x:c r="T298" t="str">
+        <x:v>https://kingpowermahanakhon.co.th/th/experience/mahanakhon-skywalk</x:v>
+      </x:c>
+      <x:c r="U298" s="23" t="str">
+        <x:v>운영사 공식 안내의 3~12세는 10:00~15:30 500바트, 15:30~19:00 600바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="36" customHeight="1">
+      <x:c r="A299" t="str">
+        <x:v>BKK-AT-009</x:v>
+      </x:c>
+      <x:c r="B299" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C299" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D299" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E299" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F299" t="str">
+        <x:v>방콕 국립박물관 외국인 개인 입장권</x:v>
+      </x:c>
+      <x:c r="G299" t="str">
+        <x:v>Bangkok National Museum Individual Admission (Foreign Visitor)</x:v>
+      </x:c>
+      <x:c r="H299" s="55" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I299" s="55" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J299" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K299" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L299" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M299" t="str">
+        <x:v>외국인 개인 방문객</x:v>
+      </x:c>
+      <x:c r="N299" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O299" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P299" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q299" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R299" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S299" t="str">
+        <x:v>Fine Arts Department, Ministry of Culture</x:v>
+      </x:c>
+      <x:c r="T299" t="str">
+        <x:v>https://www.finearts.go.th/museumnationalgallery/view/10005-%E0%B8%9A%E0%B8%B1%E0%B8%8D%E0%B8%8A%E0%B8%B5%E0%B8%84%E0%B9%88%E0%B8%B2%E0%B9%80%E0%B8%82%E0%B9%89%E0%B8%B2%E0%B8%8A%E0%B8%A1%E0%B9%82%E0%B8%9A%E0%B8%A3%E0%B8%B2%E0%B8%93%E0%B8%AA%E0%B8%96%E0%B8%B2%E0%B8%99%E0%B8%97%E0%B8%B5%E0%B9%88%E0%B9%84%E0%B8%94%E0%B9%89%E0%B8%82%E0%B8%B6%E0%B9%89%E0%B8%99%E0%B8%97%E0%B8%B0%E0%B9%80%E0%B8%9A%E0%B8%B5%E0%B8%A2%E0%B8%99%E0%B9%81%E0%B8%A5%E0%B8%B0%E0%B8%9E%E0%B8%B4%E0%B8%9E%E0%B8%B4%E0%B8%98%E0%B8%A0%E0%B8%B1%E0%B8%93%E0%B8%91%E0%B8%AA%E0%B8%96%E0%B8%B2%E0%B8%99%E0%B9%81%E0%B8%AB%E0%B9%88%E0%B8%87%E0%B8%8A%E0%B8%B2%E0%B8%95%E0%B8%B4</x:v>
+      </x:c>
+      <x:c r="U299" s="23" t="str">
+        <x:v>กรมศิลปากรระบุพิพิธภัณฑสถานแห่งชาติพระนคร ค่าเข้าชมรายบุคคลสำหรับสัญชาติอื่น 200 บาท.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="36" customHeight="1">
+      <x:c r="A300" t="str">
+        <x:v>BKK-AT-010</x:v>
+      </x:c>
+      <x:c r="B300" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C300" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D300" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E300" t="str">
+        <x:v>미술관</x:v>
+      </x:c>
+      <x:c r="F300" t="str">
+        <x:v>방콕 국립미술관 외국인 개인 입장권</x:v>
+      </x:c>
+      <x:c r="G300" t="str">
+        <x:v>Bangkok National Gallery Individual Admission (Foreign Visitor)</x:v>
+      </x:c>
+      <x:c r="H300" s="55" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I300" s="55" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J300" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K300" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L300" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M300" t="str">
+        <x:v>외국인 개인 방문객</x:v>
+      </x:c>
+      <x:c r="N300" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O300" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P300" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q300" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R300" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S300" t="str">
+        <x:v>Fine Arts Department, Ministry of Culture</x:v>
+      </x:c>
+      <x:c r="T300" t="str">
+        <x:v>https://www.finearts.go.th/museumnationalgallery/view/10005-%E0%B8%9A%E0%B8%B1%E0%B8%8D%E0%B8%8A%E0%B8%B5%E0%B8%84%E0%B9%88%E0%B8%B2%E0%B9%80%E0%B8%82%E0%B9%89%E0%B8%B2%E0%B8%8A%E0%B8%A1%E0%B9%82%E0%B8%9A%E0%B8%A3%E0%B8%B2%E0%B8%93%E0%B8%AA%E0%B8%96%E0%B8%B2%E0%B8%99%E0%B8%97%E0%B8%B5%E0%B9%88%E0%B9%84%E0%B8%94%E0%B9%89%E0%B8%82%E0%B8%B6%E0%B9%89%E0%B8%99%E0%B8%97%E0%B%B0%E0%B9%80%E0%B8%9A%E0%B8%B5%E0%B8%A2%E0%B8%99%E0%B9%81%E0%B8%A5%E0%B8%B0%E0%B8%9E%E0%B8%B4%E0%B8%9E%E0%B8%B4%E0%B8%98%E0%B8%A0%E0%B8%B1%E0%B8%93%E0%B8%91%E0%B8%AA%E0%B8%96%E0%B8%B2%E0%B8%99%E0%B9%81%E0%B8%AB%E0%B9%88%E0%B8%87%E0%B8%8A%E0%B8%B2%E0%B8%95%E0%B8%B4</x:v>
+      </x:c>
+      <x:c r="U300" s="23" t="str">
+        <x:v>กรมศิลปากรระบุพิพิธภัณฑสถานแห่งชาติหอศิลป ค่าเข้าชมรายบุคคลสำหรับสัญชาติอื่น 200 บาท.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="36" customHeight="1">
+      <x:c r="A301" t="str">
+        <x:v>BKK-AT-011</x:v>
+      </x:c>
+      <x:c r="B301" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C301" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D301" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E301" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F301" t="str">
+        <x:v>뮤지엄 시암 외국인 성인 입장권</x:v>
+      </x:c>
+      <x:c r="G301" t="str">
+        <x:v>Museum Siam Foreign Adult Admission</x:v>
+      </x:c>
+      <x:c r="H301" s="55" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I301" s="55" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J301" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K301" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L301" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M301" t="str">
+        <x:v>외국인 성인</x:v>
+      </x:c>
+      <x:c r="N301" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O301" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P301" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q301" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R301" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S301" t="str">
+        <x:v>Museum Siam</x:v>
+      </x:c>
+      <x:c r="T301" t="str">
+        <x:v>https://museumsiam.org/museumsiam-visit.php</x:v>
+      </x:c>
+      <x:c r="U301" s="23" t="str">
+        <x:v>박물관 공식 방문 안내의 외국인 성인 입장료 100바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="36" customHeight="1">
+      <x:c r="A302" t="str">
+        <x:v>BKK-AT-012</x:v>
+      </x:c>
+      <x:c r="B302" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C302" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D302" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E302" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F302" t="str">
+        <x:v>뮤지엄 시암 15세 미만 무료 입장</x:v>
+      </x:c>
+      <x:c r="G302" t="str">
+        <x:v>Museum Siam Free Admission (Under 15)</x:v>
+      </x:c>
+      <x:c r="H302" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I302" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J302" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K302" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L302" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M302" t="str">
+        <x:v>15세 미만</x:v>
+      </x:c>
+      <x:c r="N302" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O302" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P302" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q302" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R302" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S302" t="str">
+        <x:v>Museum Siam</x:v>
+      </x:c>
+      <x:c r="T302" t="str">
+        <x:v>https://museumsiam.org/museumsiam-visit.php</x:v>
+      </x:c>
+      <x:c r="U302" s="23" t="str">
+        <x:v>박물관 공식 방문 안내의 태국·외국인 15세 미만 무료 입장.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="36" customHeight="1">
+      <x:c r="A303" t="str">
+        <x:v>BKK-AT-013</x:v>
+      </x:c>
+      <x:c r="B303" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C303" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D303" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E303" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F303" t="str">
+        <x:v>방콕 플라네타리움 성인 입장권</x:v>
+      </x:c>
+      <x:c r="G303" t="str">
+        <x:v>Bangkok Planetarium Adult Admission</x:v>
+      </x:c>
+      <x:c r="H303" s="55" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I303" s="55" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J303" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K303" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L303" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M303" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N303" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O303" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P303" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q303" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R303" t="str">
+        <x:v>2026년 요금표</x:v>
+      </x:c>
+      <x:c r="S303" t="str">
+        <x:v>Science Centre for Education, Thailand</x:v>
+      </x:c>
+      <x:c r="T303" t="str">
+        <x:v>https://sciplanet.org/wp-content/uploads/2026/01/%E0%B8%AD-%E0%B9%80%E0%B8%AD%E0%B8%99%E0%B8%81%E0%B8%9B%E0%B8%A3%E0%B8%B1%E0%B8%9A-21-%E0%B8%A1.%E0%B8%84.69-%E0%B9%80%E0%B8%A5%E0%B9%88%E0%B8%A1-2569-%E0%B8%A5%E0%B9%88%E0%B8%B2%E0%B8%AA%E0%B8%B8%E0%B8%94.pdf</x:v>
+      </x:c>
+      <x:c r="U303" s="23" t="str">
+        <x:v>운영 기관의 2026년 공식 요금표상 플라네타리움 1회 성인권 50바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="36" customHeight="1">
+      <x:c r="A304" t="str">
+        <x:v>BKK-AT-014</x:v>
+      </x:c>
+      <x:c r="B304" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C304" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D304" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E304" t="str">
+        <x:v>박물관</x:v>
+      </x:c>
+      <x:c r="F304" t="str">
+        <x:v>방콕 플라네타리움 어린이 입장권</x:v>
+      </x:c>
+      <x:c r="G304" t="str">
+        <x:v>Bangkok Planetarium Child Admission</x:v>
+      </x:c>
+      <x:c r="H304" s="55" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I304" s="55" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J304" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K304" t="str">
+        <x:v>아동 1인</x:v>
+      </x:c>
+      <x:c r="L304" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M304" t="str">
+        <x:v>아동</x:v>
+      </x:c>
+      <x:c r="N304" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O304" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P304" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q304" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R304" t="str">
+        <x:v>2026년 요금표</x:v>
+      </x:c>
+      <x:c r="S304" t="str">
+        <x:v>Science Centre for Education, Thailand</x:v>
+      </x:c>
+      <x:c r="T304" t="str">
+        <x:v>https://sciplanet.org/wp-content/uploads/2026/01/%E0%B8%AD-%E0%B9%80%E0%B8%AD%E0%B8%99%E0%B8%81%E0%B8%9B%E0%B8%A3%E0%B8%B1%E0%B8%9A-21-%E0%B8%A1.%E0%B8%84.69-%E0%B9%80%E0%B8%A5%E0%B9%88%E0%B8%A1-2569-%E0%B8%A5%E0%B9%88%E0%B8%B2%E0%B8%AA%E0%B8%B8%E0%B8%94.pdf</x:v>
+      </x:c>
+      <x:c r="U304" s="23" t="str">
+        <x:v>운영 기관의 2026년 공식 요금표상 플라네타리움 어린이권 30바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="36" customHeight="1">
+      <x:c r="A305" t="str">
+        <x:v>BKK-AT-015</x:v>
+      </x:c>
+      <x:c r="B305" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C305" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D305" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E305" t="str">
+        <x:v>미술관</x:v>
+      </x:c>
+      <x:c r="F305" t="str">
+        <x:v>방콕 예술문화센터 일반 전시 입장</x:v>
+      </x:c>
+      <x:c r="G305" t="str">
+        <x:v>Bangkok Art and Culture Centre General Exhibition Admission</x:v>
+      </x:c>
+      <x:c r="H305" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I305" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J305" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K305" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L305" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M305" t="str">
+        <x:v>일반 (특별행사 제외)</x:v>
+      </x:c>
+      <x:c r="N305" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O305" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P305" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q305" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R305" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S305" t="str">
+        <x:v>Bangkok Art and Culture Centre</x:v>
+      </x:c>
+      <x:c r="T305" t="str">
+        <x:v>https://www.bacc.or.th/en/plan-your-visit</x:v>
+      </x:c>
+      <x:c r="U305" s="23" t="str">
+        <x:v>운영 기관 공식 안내: 일반 전시 무료, 특별 행사·공연은 별도 요금.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="36" customHeight="1">
+      <x:c r="A306" t="str">
+        <x:v>BKK-AT-016</x:v>
+      </x:c>
+      <x:c r="B306" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C306" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D306" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E306" t="str">
+        <x:v>정원</x:v>
+      </x:c>
+      <x:c r="F306" t="str">
+        <x:v>룸피니 공원 입장</x:v>
+      </x:c>
+      <x:c r="G306" t="str">
+        <x:v>Lumphini Park Admission</x:v>
+      </x:c>
+      <x:c r="H306" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I306" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J306" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K306" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L306" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M306" t="str">
+        <x:v>일반</x:v>
+      </x:c>
+      <x:c r="N306" t="str">
+        <x:v>B 공공</x:v>
+      </x:c>
+      <x:c r="O306" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P306" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q306" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R306" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S306" t="str">
+        <x:v>Bangkok Metropolitan Administration, Greener Bangkok</x:v>
+      </x:c>
+      <x:c r="T306" t="str">
+        <x:v>https://greener.bangkok.go.th/en/park/suan-lumpini/</x:v>
+      </x:c>
+      <x:c r="U306" s="23" t="str">
+        <x:v>방콕시 공원 안내의 입장료 무료 표기.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="36" customHeight="1">
+      <x:c r="A307" t="str">
+        <x:v>BKK-AT-017</x:v>
+      </x:c>
+      <x:c r="B307" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C307" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D307" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E307" t="str">
+        <x:v>미술관</x:v>
+      </x:c>
+      <x:c r="F307" t="str">
+        <x:v>MOCA 방콕 일반 성인 입장권</x:v>
+      </x:c>
+      <x:c r="G307" t="str">
+        <x:v>MOCA Bangkok General Adult Admission</x:v>
+      </x:c>
+      <x:c r="H307" s="55" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="I307" s="55" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="J307" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K307" t="str">
+        <x:v>성인 1인</x:v>
+      </x:c>
+      <x:c r="L307" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M307" t="str">
+        <x:v>성인</x:v>
+      </x:c>
+      <x:c r="N307" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O307" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P307" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q307" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R307" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S307" t="str">
+        <x:v>Museum of Contemporary Art Bangkok</x:v>
+      </x:c>
+      <x:c r="T307" t="str">
+        <x:v>https://www.mocabangkok.com/admission/</x:v>
+      </x:c>
+      <x:c r="U307" s="23" t="str">
+        <x:v>미술관 공식 일반 입장권 성인 요금 400바트.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="36" customHeight="1">
+      <x:c r="A308" t="str">
+        <x:v>BKK-AT-018</x:v>
+      </x:c>
+      <x:c r="B308" t="str">
+        <x:v>태국</x:v>
+      </x:c>
+      <x:c r="C308" t="str">
+        <x:v>방콕</x:v>
+      </x:c>
+      <x:c r="D308" t="str">
+        <x:v>관광</x:v>
+      </x:c>
+      <x:c r="E308" t="str">
+        <x:v>미술관</x:v>
+      </x:c>
+      <x:c r="F308" t="str">
+        <x:v>MOCA 방콕 13세 미만 무료 입장</x:v>
+      </x:c>
+      <x:c r="G308" t="str">
+        <x:v>MOCA Bangkok Free Admission (Under 13)</x:v>
+      </x:c>
+      <x:c r="H308" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I308" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J308" t="str">
+        <x:v>THB</x:v>
+      </x:c>
+      <x:c r="K308" t="str">
+        <x:v>1인</x:v>
+      </x:c>
+      <x:c r="L308" t="str">
+        <x:v>고정형</x:v>
+      </x:c>
+      <x:c r="M308" t="str">
+        <x:v>13세 미만</x:v>
+      </x:c>
+      <x:c r="N308" t="str">
+        <x:v>A 공식</x:v>
+      </x:c>
+      <x:c r="O308" t="str">
+        <x:v>예</x:v>
+      </x:c>
+      <x:c r="P308" t="str">
+        <x:v>확정 1차</x:v>
+      </x:c>
+      <x:c r="Q308" s="51" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="R308" t="str">
+        <x:v>2026-10-03 확인</x:v>
+      </x:c>
+      <x:c r="S308" t="str">
+        <x:v>Museum of Contemporary Art Bangkok</x:v>
+      </x:c>
+      <x:c r="T308" t="str">
+        <x:v>https://www.mocabangkok.com/admission/</x:v>
+      </x:c>
+      <x:c r="U308" s="23" t="str">
+        <x:v>미술관 공식 일반 입장 안내의 13세 미만 무료.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:U1"/>
@@ -20703,7 +21678,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ef03347cb3b41b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b625a6860834773"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22422,7 +23397,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5df684e6f7994c98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03176ac2d89940e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23494,7 +24469,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b0c1d232c041c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6c1913005384b05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>